<commit_message>
ajout des liens ecoles
</commit_message>
<xml_diff>
--- a/parametres_simulateur_inphb.xlsx
+++ b/parametres_simulateur_inphb.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0bc125c4368f47fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coefficients_bac" sheetId="2" r:id="Rf8abc7dcda8b4179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coefficients_inphb" sheetId="3" r:id="R32474a34932142c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eligibilite_inphb" sheetId="4" r:id="R39ed76f6340b45b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="places_estimees" sheetId="5" r:id="R275ffc48bf6544ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mentions_inphb" sheetId="6" r:id="Rce537ed17caf48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stats_series_2025" sheetId="7" r:id="Re21e8c81ada0440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groupes_matieres" sheetId="8" r:id="R3d95fceb73e4425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R00e36fb9fed24cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coefficients_bac" sheetId="2" r:id="Ra878fc66adcb4ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coefficients_inphb" sheetId="3" r:id="Radd5faa3790b47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eligibilite_inphb" sheetId="4" r:id="R28ded44607bd4160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="places_estimees" sheetId="5" r:id="R291c1041482d4331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mentions_inphb" sheetId="6" r:id="Rab0bf131908a4e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stats_series_2025" sheetId="7" r:id="Re403d86b53fb4a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="groupes_matieres" sheetId="8" r:id="R9577b12d26e44cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liens_filieres" sheetId="9" r:id="Rf9716bd00cb14b0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -702,7 +703,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -739,9 +740,42 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF123B5D"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="9">
     <x:border diagonalUp="0" diagonalDown="0"/>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left/>
+      <x:top/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right/>
+      <x:top/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left/>
+      <x:bottom/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:bottom/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right/>
+      <x:bottom/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="26">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -775,7 +809,7 @@
     </x:xf>
     <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="47">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -862,6 +896,60 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="12">
@@ -4276,7 +4364,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R164ed97395804641"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc40af47fe8b4be6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8122,7 +8210,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ea01c806254178"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae0b812ea0447b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9229,7 +9317,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40fd5fc8068a4c89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R815e67d27ee24e50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10254,7 +10342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ef610a289134f65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree55753f34fe4d64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11104,7 +11192,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f2b5a732fc342a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102caef4985c4757"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12296,7 +12384,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb6216296fe48af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb6d4a5fe3c14c82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14556,4 +14644,390 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="38" t="str">
+        <x:v>filiere</x:v>
+      </x:c>
+      <x:c r="B1" s="39" t="str">
+        <x:v>ecole</x:v>
+      </x:c>
+      <x:c r="C1" s="39" t="str">
+        <x:v>cycle</x:v>
+      </x:c>
+      <x:c r="D1" s="39" t="str">
+        <x:v>intitule</x:v>
+      </x:c>
+      <x:c r="E1" s="39" t="str">
+        <x:v>url_officielle</x:v>
+      </x:c>
+      <x:c r="F1" s="39" t="str">
+        <x:v>type_lien</x:v>
+      </x:c>
+      <x:c r="G1" s="40" t="str">
+        <x:v>commentaire</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="41" t="str">
+        <x:v>GAE</x:v>
+      </x:c>
+      <x:c r="B2" s="42" t="str">
+        <x:v>ESCAE</x:v>
+      </x:c>
+      <x:c r="C2" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D2" s="42" t="str">
+        <x:v>Gestion appliquée aux entreprises</x:v>
+      </x:c>
+      <x:c r="E2" s="42" t="str">
+        <x:v>https://escae.inphb.ci/public/formations</x:v>
+      </x:c>
+      <x:c r="F2" s="42" t="str">
+        <x:v>Page de l'école</x:v>
+      </x:c>
+      <x:c r="G2" s="43" t="str">
+        <x:v>Offre de formation officielle de l'ESCAE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="41" t="str">
+        <x:v>FCA</x:v>
+      </x:c>
+      <x:c r="B3" s="42" t="str">
+        <x:v>ESCAE</x:v>
+      </x:c>
+      <x:c r="C3" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D3" s="42" t="str">
+        <x:v>Finance, comptabilité et audit</x:v>
+      </x:c>
+      <x:c r="E3" s="42" t="str">
+        <x:v>https://escae.inphb.ci/public/formations</x:v>
+      </x:c>
+      <x:c r="F3" s="42" t="str">
+        <x:v>Page de l'école</x:v>
+      </x:c>
+      <x:c r="G3" s="43" t="str">
+        <x:v>Offre de formation officielle de l'ESCAE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="41" t="str">
+        <x:v>ECG</x:v>
+      </x:c>
+      <x:c r="B4" s="42" t="str">
+        <x:v>CPGE</x:v>
+      </x:c>
+      <x:c r="C4" s="42" t="str">
+        <x:v>Cycle préparatoire</x:v>
+      </x:c>
+      <x:c r="D4" s="42" t="str">
+        <x:v>Économique et commerciale générale</x:v>
+      </x:c>
+      <x:c r="E4" s="42" t="str">
+        <x:v>https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</x:v>
+      </x:c>
+      <x:c r="F4" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G4" s="43" t="str">
+        <x:v>Plaquette officielle des classes préparatoires de l'INP-HB.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="41" t="str">
+        <x:v>BCPST</x:v>
+      </x:c>
+      <x:c r="B5" s="42" t="str">
+        <x:v>CPGE</x:v>
+      </x:c>
+      <x:c r="C5" s="42" t="str">
+        <x:v>Cycle préparatoire</x:v>
+      </x:c>
+      <x:c r="D5" s="42" t="str">
+        <x:v>Biologie, chimie, physique et sciences de la Terre</x:v>
+      </x:c>
+      <x:c r="E5" s="42" t="str">
+        <x:v>https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</x:v>
+      </x:c>
+      <x:c r="F5" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G5" s="43" t="str">
+        <x:v>Plaquette officielle des classes préparatoires de l'INP-HB.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="41" t="str">
+        <x:v>MPSI</x:v>
+      </x:c>
+      <x:c r="B6" s="42" t="str">
+        <x:v>CPGE</x:v>
+      </x:c>
+      <x:c r="C6" s="42" t="str">
+        <x:v>Cycle préparatoire</x:v>
+      </x:c>
+      <x:c r="D6" s="42" t="str">
+        <x:v>Mathématiques, physique et sciences de l'ingénieur</x:v>
+      </x:c>
+      <x:c r="E6" s="42" t="str">
+        <x:v>https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</x:v>
+      </x:c>
+      <x:c r="F6" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G6" s="43" t="str">
+        <x:v>Plaquette officielle des classes préparatoires de l'INP-HB.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>MP2I</x:v>
+      </x:c>
+      <x:c r="B7" s="42" t="str">
+        <x:v>CPGE</x:v>
+      </x:c>
+      <x:c r="C7" s="42" t="str">
+        <x:v>Cycle préparatoire</x:v>
+      </x:c>
+      <x:c r="D7" s="42" t="str">
+        <x:v>Mathématiques, physique, ingénierie et informatique</x:v>
+      </x:c>
+      <x:c r="E7" s="42" t="str">
+        <x:v>https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</x:v>
+      </x:c>
+      <x:c r="F7" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G7" s="43" t="str">
+        <x:v>Lien vers la présentation officielle des classes préparatoires ; la plaquette publiée peut ne pas détailler cette voie récente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="41" t="str">
+        <x:v>PCSI</x:v>
+      </x:c>
+      <x:c r="B8" s="42" t="str">
+        <x:v>CPGE</x:v>
+      </x:c>
+      <x:c r="C8" s="42" t="str">
+        <x:v>Cycle préparatoire</x:v>
+      </x:c>
+      <x:c r="D8" s="42" t="str">
+        <x:v>Physique, chimie et sciences de l'ingénieur</x:v>
+      </x:c>
+      <x:c r="E8" s="42" t="str">
+        <x:v>https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</x:v>
+      </x:c>
+      <x:c r="F8" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G8" s="43" t="str">
+        <x:v>Lien vers la présentation officielle des classes préparatoires ; la plaquette publiée peut ne pas détailler cette voie récente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="41" t="str">
+        <x:v>TSA</x:v>
+      </x:c>
+      <x:c r="B9" s="42" t="str">
+        <x:v>ESA</x:v>
+      </x:c>
+      <x:c r="C9" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D9" s="42" t="str">
+        <x:v>Technicien supérieur en agronomie</x:v>
+      </x:c>
+      <x:c r="E9" s="42" t="str">
+        <x:v>https://inphb.ci/static/media/ESA.1e3e6705a0c038fbfec7.pdf</x:v>
+      </x:c>
+      <x:c r="F9" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G9" s="43" t="str">
+        <x:v>Plaquette officielle de l'École supérieure d'agronomie.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="41" t="str">
+        <x:v>STIC</x:v>
+      </x:c>
+      <x:c r="B10" s="42" t="str">
+        <x:v>ESI</x:v>
+      </x:c>
+      <x:c r="C10" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="str">
+        <x:v>Sciences et technologies de l'information et de la communication</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="str">
+        <x:v>https://inphb.ci/static/media/ESI.6d5a13044a0918a30dd7.pdf</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G10" s="43" t="str">
+        <x:v>Plaquette officielle de l'École supérieure d'industrie.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="41" t="str">
+        <x:v>STGI</x:v>
+      </x:c>
+      <x:c r="B11" s="42" t="str">
+        <x:v>ESI</x:v>
+      </x:c>
+      <x:c r="C11" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D11" s="42" t="str">
+        <x:v>Sciences et technologies du génie industriel</x:v>
+      </x:c>
+      <x:c r="E11" s="42" t="str">
+        <x:v>https://inphb.ci/static/media/ESI.6d5a13044a0918a30dd7.pdf</x:v>
+      </x:c>
+      <x:c r="F11" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G11" s="43" t="str">
+        <x:v>Plaquette officielle de l'École supérieure d'industrie.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="41" t="str">
+        <x:v>GC</x:v>
+      </x:c>
+      <x:c r="B12" s="42" t="str">
+        <x:v>ESTP</x:v>
+      </x:c>
+      <x:c r="C12" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D12" s="42" t="str">
+        <x:v>Génie civil</x:v>
+      </x:c>
+      <x:c r="E12" s="42" t="str">
+        <x:v>https://inphb.ci/static/media/ESTP.fc83b695d74550741d9b.pdf</x:v>
+      </x:c>
+      <x:c r="F12" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G12" s="43" t="str">
+        <x:v>Plaquette officielle de l'École supérieure des travaux publics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="41" t="str">
+        <x:v>MG</x:v>
+      </x:c>
+      <x:c r="B13" s="42" t="str">
+        <x:v>ESMG</x:v>
+      </x:c>
+      <x:c r="C13" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D13" s="42" t="str">
+        <x:v>Mines et géologie</x:v>
+      </x:c>
+      <x:c r="E13" s="42" t="str">
+        <x:v>https://inphb.ci/static/media/ESMG.3673dcbd14528ad175ac.pdf</x:v>
+      </x:c>
+      <x:c r="F13" s="42" t="str">
+        <x:v>Plaquette officielle</x:v>
+      </x:c>
+      <x:c r="G13" s="43" t="str">
+        <x:v>Plaquette officielle de l'École supérieure des mines et de géologie.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="41" t="str">
+        <x:v>PME</x:v>
+      </x:c>
+      <x:c r="B14" s="42" t="str">
+        <x:v>ESCPE</x:v>
+      </x:c>
+      <x:c r="C14" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D14" s="42" t="str">
+        <x:v>Procédés et maîtrise de l'énergie</x:v>
+      </x:c>
+      <x:c r="E14" s="42" t="str">
+        <x:v>https://www.inphb.ci/</x:v>
+      </x:c>
+      <x:c r="F14" s="42" t="str">
+        <x:v>Site officiel INP-HB</x:v>
+      </x:c>
+      <x:c r="G14" s="43" t="str">
+        <x:v>Aucune fiche publique stable et spécifique n'a été identifiée ; lien vers le site officiel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="41" t="str">
+        <x:v>CGP</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="str">
+        <x:v>ESCPE</x:v>
+      </x:c>
+      <x:c r="C15" s="42" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D15" s="42" t="str">
+        <x:v>Chimie et génie des procédés</x:v>
+      </x:c>
+      <x:c r="E15" s="42" t="str">
+        <x:v>https://www.inphb.ci/</x:v>
+      </x:c>
+      <x:c r="F15" s="42" t="str">
+        <x:v>Site officiel INP-HB</x:v>
+      </x:c>
+      <x:c r="G15" s="43" t="str">
+        <x:v>Aucune fiche publique stable et spécifique n'a été identifiée ; lien vers le site officiel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="44" t="str">
+        <x:v>TSAERO</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>ESAS</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>Cycle court</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="str">
+        <x:v>Technicien supérieur aéronautique</x:v>
+      </x:c>
+      <x:c r="E16" s="45" t="str">
+        <x:v>https://www.inphb.ci/</x:v>
+      </x:c>
+      <x:c r="F16" s="45" t="str">
+        <x:v>Site officiel INP-HB</x:v>
+      </x:c>
+      <x:c r="G16" s="46" t="str">
+        <x:v>Aucune fiche publique stable et spécifique n'a été identifiée ; lien vers le site officiel.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
nettoyage et correction des liens
</commit_message>
<xml_diff>
--- a/parametres_simulateur_inphb.xlsx
+++ b/parametres_simulateur_inphb.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -813,7 +813,7 @@
     <t xml:space="preserve">Gestion appliquée aux entreprises</t>
   </si>
   <si>
-    <t xml:space="preserve">https://escae.inphb.ci/public/formations</t>
+    <t xml:space="preserve">https://escae.inphb.ci/public/formations/cycle-technicien-superieur</t>
   </si>
   <si>
     <t xml:space="preserve">Page de l'école</t>
@@ -834,7 +834,7 @@
     <t xml:space="preserve">Économique et commerciale générale</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.inphb.ci/static/media/CPGE.9b4d786a11dd59ac7ac1.pdf</t>
+    <t xml:space="preserve">https://inphb.edu.ci/nos-ecoles/cpge/filieres/</t>
   </si>
   <si>
     <t xml:space="preserve">Plaquette officielle</t>
@@ -900,7 +900,7 @@
     <t xml:space="preserve">Procédés et maîtrise de l'énergie</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.inphb.ci/</t>
+    <t xml:space="preserve">https://inphb.edu.ci/nos-ecoles/</t>
   </si>
   <si>
     <t xml:space="preserve">Site officiel INP-HB</t>

</xml_diff>